<commit_message>
scan: seg6 2026-10-26 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq7_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>66.13921077791568</v>
+        <v>66.1392107296813</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>38.17180851254412</v>
+        <v>38.17180869844601</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.783462123423861</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.3898117229241027</v>
+        <v>0.3898117225347661</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>67.9930128536185</v>
+        <v>67.99301297688395</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>33.76309478282229</v>
+        <v>33.76309485096934</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.16131508790875</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.909568500168254</v>
+        <v>2.909568498481043</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>59.43460120810688</v>
+        <v>59.43460131000813</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>32.95138989656964</v>
+        <v>32.95138991962353</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.8531135934803761</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.3295393360125356</v>
+        <v>0.3295393344551192</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.45357814780608</v>
+        <v>65.45357812491665</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>42.47737227737745</v>
+        <v>42.47737231439886</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.9817295434887761</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.9360722877392078</v>
+        <v>0.9360722867009024</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>59.26265204435855</v>
+        <v>59.26265219171178</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23.4359230842435</v>
+        <v>23.43592318906657</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.590262182470743</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.4499754979033113</v>
+        <v>0.4499754969948003</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>78.84064550548312</v>
+        <v>78.84064557796489</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>28.03469081350088</v>
+        <v>28.03469086900749</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.805710472882409</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3.452091477781269</v>
+        <v>3.452091477314043</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>772.9581839293658</v>
+        <v>772.9581839293656</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>778</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>53.54270781241167</v>
+        <v>53.54270783774406</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>33.66656639699555</v>
+        <v>33.66656639386537</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.6014135830005847</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-8.764929623296041</v>
+        <v>-8.764929627189638</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65.62661536390686</v>
+        <v>65.62661536859808</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>62.72758503336988</v>
+        <v>62.72758505166355</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.016111572061801</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>4.675131239069174</v>
+        <v>4.675131238420221</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>707.6393411866204</v>
+        <v>707.6393411866211</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>30.3</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>66.18318996901441</v>
+        <v>66.18319005050003</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>18.52913189178017</v>
+        <v>18.52913199507876</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.639202115466247</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2807110429879311</v>
+        <v>0.2807110429230415</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>52.83820007593084</v>
+        <v>52.83820016037561</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>27.74815458778912</v>
+        <v>27.7481548157389</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.7489979191491927</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-14.95427630484705</v>
+        <v>-14.9542763334002</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>54.83324439766531</v>
+        <v>54.83324439600781</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>57.22228090028041</v>
+        <v>57.22228095341231</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.8508086301746604</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.8708864216365662</v>
+        <v>-0.870886421714447</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>58.46748194742087</v>
+        <v>58.46748228248495</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>29.42322240553066</v>
+        <v>29.42322241829411</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.4228143041877703</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.2813739001872606</v>
+        <v>-0.2813739006544933</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>54.44818794913423</v>
+        <v>54.44818794517776</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>30.82920262634143</v>
+        <v>30.82920264781097</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.9635624771200302</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-5.137034637696825</v>
+        <v>-5.137034638345732</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>43.35024341495217</v>
+        <v>43.35024341425321</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>27.30615665604493</v>
+        <v>27.30615659592426</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.5381821608099771</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-9.710584682145402</v>
+        <v>-9.710584682508859</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.86263548571269</v>
+        <v>51.8626354899997</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>48.28267896357842</v>
+        <v>48.28267928124164</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.569845152521627</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-1.284393853037365</v>
+        <v>-1.284393853309933</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>50.18528358627345</v>
+        <v>50.18528360302879</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>39.06509006749615</v>
+        <v>39.06509014432356</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4366239614420854</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-1.414578922257699</v>
+        <v>-1.414578922880661</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46.79904150441659</v>
+        <v>46.79904153805073</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15.97781206326698</v>
+        <v>15.97781209733668</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.7493361150785418</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-15.21772423639853</v>
+        <v>-15.217724242888</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>43.07886113082659</v>
+        <v>43.07886121885245</v>
       </c>
       <c r="I19" s="2" t="n">
         <v>23.76290932082123</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-11.26967931245293</v>
+        <v>-11.26967931414019</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>68.41252457395312</v>
+        <v>68.41252470798648</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>36.23932810385143</v>
+        <v>36.2393281840283</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.71445693349921</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>1.092136652482862</v>
+        <v>1.09213665188584</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>53.34021957175199</v>
+        <v>53.34021960790697</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>46.52032355701385</v>
+        <v>46.52032367085199</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.6871215099514526</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.4374775598750293</v>
+        <v>-0.437477560446089</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.48352340529029</v>
+        <v>51.48352346686449</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>50.23478165147062</v>
+        <v>50.23478175815763</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.6979013411604504</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.2186659809617515</v>
+        <v>-0.2186659814809033</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>31.69496627512719</v>
+        <v>31.69503670044691</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>32.59378792018985</v>
+        <v>32.59384563926454</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>2.013053626871307</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.4112802574506249</v>
+        <v>0.4112800741141505</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>44.81020337513287</v>
+        <v>44.81020338410932</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>40.69951888017797</v>
+        <v>40.69951900598078</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.4716996868395078</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-2.284573292876708</v>
+        <v>-2.284573293188202</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>502.5889994943346</v>
+        <v>502.5889994943347</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>311.5</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>47.37589237653724</v>
+        <v>47.37589240126501</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>14.92085523866844</v>
+        <v>14.92085526119895</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.106793234680007</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.7874918210217718</v>
+        <v>0.7874918208919892</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.3834705294757</v>
+        <v>51.38347057721097</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>27.49474097369329</v>
+        <v>27.49474112937997</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7258430839794561</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.462579100670226</v>
+        <v>0.4625791000991539</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>54.78509627337731</v>
+        <v>54.78509626425939</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>27.82618268687443</v>
+        <v>27.82618267411424</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.132039438032072</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.9246587922949843</v>
+        <v>-0.9246587924377483</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>490.6030553005186</v>
+        <v>490.6030553005187</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>135</v>
@@ -1933,7 +1933,7 @@
         <v>53.56737410844026</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>9.652436747216374</v>
+        <v>9.652436801055186</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.2573020601650947</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2.051568861571004</v>
+        <v>2.051568861311428</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.34519234929413</v>
+        <v>56.34519241469733</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.05654013574955</v>
+        <v>28.056540362229</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.025511535086557</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.1872518388045469</v>
+        <v>0.1872518385968903</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>52.88280136246697</v>
+        <v>52.88280168553795</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>5.805251238055731</v>
+        <v>5.805252003337797</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>7.041140377347645</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.306921393108382</v>
+        <v>1.306921375327576</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>52.05564347176647</v>
+        <v>52.0556434529181</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.29868578151176</v>
+        <v>26.2986858100039</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.8608248155283107</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.01786095518375885</v>
+        <v>-0.01786095505396873</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>472.1137159469964</v>
+        <v>472.113715946996</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>252</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.82436373612074</v>
+        <v>44.82436370508728</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.81613424033785</v>
+        <v>31.81613439668219</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.3268196648928203</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-3.159187635293017</v>
+        <v>-3.159187638148364</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>469.5593099855826</v>
+        <v>469.5593099855828</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>73.5</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>43.73114175472426</v>
+        <v>43.73114175639572</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.3448784142345</v>
+        <v>26.34487843277425</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.6504221412525585</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.5703199971197042</v>
+        <v>-0.5703199971067308</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>56.3009076786227</v>
+        <v>56.3009077493245</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>51.7672816331941</v>
+        <v>51.76728172823847</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.7293381745137858</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.5204985935676736</v>
+        <v>-0.5204985936455411</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>43.0338197257606</v>
+        <v>43.03381971953389</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>12.36682419601254</v>
+        <v>12.36682424409357</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.083874176340649</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.8400575301394879</v>
+        <v>-0.8400575301784277</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>43.18350452902783</v>
+        <v>43.1835045825207</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>12.40643352193912</v>
+        <v>12.40643357572483</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6707571425321006</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.2985029108869748</v>
+        <v>-0.2985029117954729</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>430.2730399096471</v>
+        <v>430.2730399096475</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>33.35</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>51.72229193807957</v>
+        <v>51.72229192552977</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>9.070079206201751</v>
+        <v>9.070079142315496</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.3094123228614452</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.673130596577153</v>
+        <v>0.6731305966550249</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>426.6714799216061</v>
+        <v>426.6714799216026</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>438</v>
@@ -2463,7 +2463,7 @@
         <v>43.4631689606963</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>16.89368722054554</v>
+        <v>16.89368721941255</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.345272722820805</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-3.835548447691353</v>
+        <v>-3.835548446912627</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>408.0379727000432</v>
+        <v>408.0379727000433</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>200</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46.49124109693207</v>
+        <v>46.49124106814377</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>24.15841561756872</v>
+        <v>24.1584157632592</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3055407865693525</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-2.150556973802361</v>
+        <v>-2.150556973750456</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>405.7485851320558</v>
+        <v>405.7485851320556</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>20.25</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>51.94049266944791</v>
+        <v>51.94049266350598</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>7.008650154560302</v>
+        <v>7.008649904222151</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.2940991325586373</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.4766114651012215</v>
+        <v>0.4766114651531362</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.95463244861767</v>
+        <v>66.95463226293367</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>45.75795671080839</v>
+        <v>45.75795694778152</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.02373845207331912</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.0821077122519589</v>
+        <v>-0.08210771244663961</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>393.1566549990978</v>
+        <v>393.1566549990977</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>330</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>35.84716749112027</v>
+        <v>35.84716741032861</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>17.17900470099632</v>
+        <v>17.17900475190858</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.089224249952527</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-4.485548447305684</v>
+        <v>-4.485548443541893</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>46.2031630039136</v>
+        <v>46.20316293156278</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>24.30802611642499</v>
+        <v>24.30802590981961</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.8379661521848411</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.01860860959894473</v>
+        <v>-0.01860860946915094</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>48.30030406820968</v>
+        <v>48.30030412799786</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>18.16462391225805</v>
+        <v>18.16462395776582</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.5443416099734087</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.2480839147483065</v>
+        <v>-0.2480839149300026</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>375.2572561347597</v>
+        <v>375.2572561347595</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>101</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>40.09459931242485</v>
+        <v>40.09459933619632</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>18.99730022940674</v>
+        <v>18.99730027605282</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.1878142965022349</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-1.404968962617764</v>
+        <v>-1.404968961968843</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>371.6713152146872</v>
+        <v>371.6713152146871</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>15.45</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>57.95102154789164</v>
+        <v>57.95102201636346</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>31.95665099868492</v>
+        <v>31.95665076381545</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.3298076254041656</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.1895555945531584</v>
+        <v>-0.1895555951710248</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>46.72811487457408</v>
+        <v>46.72811523788231</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>11.26984681573407</v>
+        <v>11.26984672375984</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6769276009064168</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.01091292166315272</v>
+        <v>-0.01091292296101987</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>367.037025508366</v>
+        <v>367.0370255083652</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>72.3</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>48.32045142948066</v>
+        <v>48.32045144933695</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>31.32192072941047</v>
+        <v>31.32192080889711</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.2662409917239372</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.109418256143197</v>
+        <v>-1.10941825648063</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>360.4100534133017</v>
+        <v>360.4100534133018</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>78.90000000000001</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>43.56709063815178</v>
+        <v>43.56709064958579</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>10.08296178746914</v>
+        <v>10.08296175367835</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>2.549799792792541</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.1478458583063567</v>
+        <v>-0.1478458583582646</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>356.9683100161366</v>
+        <v>356.9683100161362</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>31.5</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.9265096791893</v>
+        <v>48.92650940199975</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.99380511670344</v>
+        <v>19.99380493462421</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5109288470936049</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.02340443981772056</v>
+        <v>0.02340443989559124</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>354.3485990985605</v>
+        <v>354.3485990985603</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>435</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.99051751673993</v>
+        <v>42.99051756841304</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>20.66308833271936</v>
+        <v>20.66308834710163</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.3495772391539256</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-8.01402195006176</v>
+        <v>-8.014021952917089</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>38.18810825860295</v>
+        <v>38.18810824051624</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>17.91025755383243</v>
+        <v>17.91025758856495</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.7056395626210019</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-20.7878731135776</v>
+        <v>-20.78787311305849</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>33.17659646924214</v>
+        <v>33.17659636557011</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>20.26534191537275</v>
+        <v>20.26534206916199</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5502769291013172</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.08970069856864271</v>
+        <v>0.089700698283113</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>35.37096399615106</v>
+        <v>35.37096399870065</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.63443387476046</v>
+        <v>19.63443392768182</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4854669172735663</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-4.725979832917121</v>
+        <v>-4.725979832839229</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>342.5101624727927</v>
+        <v>342.510162472793</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>13.65</v>
@@ -3361,7 +3361,7 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.50275300089988</v>
+        <v>52.50275291412495</v>
       </c>
       <c r="I55" s="2" t="n">
         <v>32.03331397758119</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.04269046723110043</v>
+        <v>0.04269046727003761</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>341.6518351144351</v>
+        <v>341.6518351144287</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>32.45</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.58701158008623</v>
+        <v>44.58701152949315</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>34.91832389867675</v>
+        <v>34.91832383570953</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6421649717445593</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.0669870700338091</v>
+        <v>-0.06698707021551151</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>49.0755861064055</v>
+        <v>49.07558613941439</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.76965330145682</v>
+        <v>29.76965326559563</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.2095738242586338</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0147037856747767</v>
+        <v>0.0147037856488178</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>337.2072573496718</v>
+        <v>337.2072573496719</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>91.2</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>45.5728460919075</v>
+        <v>45.57284605879392</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22.30864816430322</v>
+        <v>22.30864813798438</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.3985145381141949</v>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>335.8860035101117</v>
+        <v>335.8860035101118</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>454</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>34.22897737117232</v>
+        <v>34.22897735258211</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.73589112190929</v>
+        <v>20.73589107735793</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.9734623319790414</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-8.648725456362472</v>
+        <v>-8.648725455973132</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>41.14913932672835</v>
+        <v>41.14913936781046</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>25.72357658324565</v>
+        <v>25.72357658324564</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.402942734216557</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.1216434037127472</v>
+        <v>0.1216434035570048</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3682,7 +3682,7 @@
         <v>53.44229464300494</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.63202250609801</v>
+        <v>11.6320224634039</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.8362066563706447</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.08618012225904795</v>
+        <v>0.08618012212925803</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>32.50477979387696</v>
+        <v>32.50477980118534</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>23.76985614022453</v>
+        <v>23.76985613690461</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4050616365577276</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-2.111207928924443</v>
+        <v>-2.111207928976355</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.95815847630649</v>
+        <v>45.95815849138076</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.62736455016586</v>
+        <v>23.62736460384406</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.2951796718019397</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-8.083918670561296</v>
+        <v>-8.083918670691094</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>43.44051006655321</v>
+        <v>43.44051007368235</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.19302545393563</v>
+        <v>15.19302544013198</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.5672759078947981</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.02873342436623072</v>
+        <v>0.02873342428836156</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>32.35210810750007</v>
+        <v>32.35210813950101</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>16.34739219050756</v>
+        <v>16.34739219273574</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8197253114347555</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.805532682209512</v>
+        <v>-1.805532682131642</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>27.72976056923552</v>
+        <v>27.72976066393656</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>42.34235297565569</v>
+        <v>42.34235323582792</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.004128314746851</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>75.32137562471053</v>
+        <v>75.32137559096594</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>297.7362003466072</v>
+        <v>297.7362003466068</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>260</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>34.33551205898286</v>
+        <v>34.33551212391791</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>27.29241267733122</v>
+        <v>27.29241267166761</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.836939751452674</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.246964943475587</v>
+        <v>-0.2469649439947585</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>29.52310216379202</v>
+        <v>29.52310241874801</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>25.6884037064428</v>
+        <v>25.68840367579241</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.200584827670398</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-9.807987010838009</v>
+        <v>-9.807987038093273</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>279.0374276364244</v>
+        <v>279.0374276364245</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>72.5</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>38.43366157993682</v>
+        <v>38.43366142992564</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>13.86832625993961</v>
+        <v>13.86832634216873</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.7472854498730647</v>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>277.7385177368521</v>
+        <v>277.7385177368528</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>395.5</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>28.43930782194518</v>
+        <v>28.43930784168762</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>35.77449946900473</v>
+        <v>35.7744994488714</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7541966637473086</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-4.238642013442416</v>
+        <v>-4.238642015778581</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>277.3596224344001</v>
+        <v>277.3596224343956</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>58.3</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>43.39129107888872</v>
+        <v>43.39129164622928</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>35.56974150961355</v>
+        <v>35.56974151595632</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6387248817360134</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1680993623055167</v>
+        <v>-0.1680993623833887</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>276.9361253032194</v>
+        <v>276.9361253032197</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>31.7</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>47.67833437786363</v>
+        <v>47.67833461021966</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>9.788952112646465</v>
+        <v>9.78895211616444</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.5970128778915239</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.1662612067999174</v>
+        <v>-0.1662612070594894</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>276.911910842875</v>
+        <v>276.9119108428752</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>149.5</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>46.02335611755827</v>
+        <v>46.02335630685144</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.44621648324204</v>
+        <v>14.4462165566942</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7434437233323928</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.05975606571259204</v>
+        <v>-0.05975606739983655</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>29.22695805838411</v>
+        <v>29.22695765456382</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>27.55583681295032</v>
+        <v>27.55583681127679</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.7308142214645494</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.458553580742664</v>
+        <v>-1.458553579185219</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>275.0239908494919</v>
+        <v>275.0239908494917</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>441</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>26.46661254095284</v>
+        <v>26.46661251627982</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>29.81781720171369</v>
+        <v>29.81781723267084</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.8925733520485345</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-6.633611729168329</v>
+        <v>-6.633611730725779</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>268.1452942390131</v>
+        <v>268.1452942390133</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>45.8</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>40.84354961761059</v>
+        <v>40.84354946040339</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>18.44149877586604</v>
+        <v>18.4414987393686</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5938828997542779</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.3072017300932292</v>
+        <v>-0.3072017301711005</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>263.077810366472</v>
+        <v>263.0778103664687</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>30.7</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>44.23307528013046</v>
+        <v>44.23307551790457</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>10.22886679797319</v>
+        <v>10.22886681524779</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4323671099305398</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.01826863801870987</v>
+        <v>-0.0182686383042428</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>259.9620847677764</v>
+        <v>259.9620847677766</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>120</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>24.94382247134943</v>
+        <v>24.94382259600208</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>25.98054362652402</v>
+        <v>25.98054366655018</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.8455976587157367</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.66735421336604</v>
+        <v>-0.6673542159617645</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>48.58712145242531</v>
+        <v>48.58712143966925</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>8.315858922171259</v>
+        <v>8.315858922171255</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.500846362264681</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>44.84000708769018</v>
+        <v>44.84000589582177</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>11.7167494853561</v>
+        <v>11.71674973081112</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.334053863089634</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.07905838745949656</v>
+        <v>0.07905838836800649</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>244.4507352996497</v>
+        <v>244.4507352996496</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>22.7</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>43.29872308636841</v>
+        <v>43.29872271509428</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13.85678706511383</v>
+        <v>13.85678704041722</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1.862922723609504</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.002855709540098662</v>
+        <v>0.002855709708819942</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>47.19009963491568</v>
+        <v>47.19009974328522</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>46.63856798812848</v>
+        <v>46.63856802785586</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4126321019762629</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.1116978078983616</v>
+        <v>-0.11169780820985</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>228.3106571009499</v>
+        <v>228.3106571009501</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>1185</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>36.0633561033358</v>
+        <v>36.06335611145087</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.79376421006533</v>
+        <v>15.79376418230428</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.3608053483989695</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-35.14971342061607</v>
+        <v>-35.14971342308185</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>46.68799819712713</v>
+        <v>46.68799822251765</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>14.64900044434147</v>
+        <v>14.64900051592594</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3262171362946557</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.03055587939005819</v>
+        <v>0.03055587933814333</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>221.8527820116681</v>
+        <v>221.8527820116686</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>144.5</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>27.60894640375253</v>
+        <v>27.60894648873207</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>25.30617062340142</v>
+        <v>25.30617069015616</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.9479146470974632</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.598952409860657</v>
+        <v>-1.598952410509593</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>221.1790849490211</v>
+        <v>221.1790849490206</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>52.6</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>41.77962502993267</v>
+        <v>41.77962525496796</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.08018112863078</v>
+        <v>12.08018110625801</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.8521506427035332</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.01195447563781354</v>
+        <v>-0.01195447589739312</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>35.29255681073134</v>
+        <v>35.2925568095651</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>20.52550758911565</v>
+        <v>20.52550766544719</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.6771364144255658</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-31.71910484911709</v>
+        <v>-31.71910485106393</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>219.169860822402</v>
+        <v>219.1698608224019</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>93.40000000000001</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>29.57274239359724</v>
+        <v>29.57274247949711</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>38.79309219339915</v>
+        <v>38.79309213470124</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.726196054107507</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.4162327268943273</v>
+        <v>-0.4162327281921847</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>216.7999481026542</v>
+        <v>216.7999481026544</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>48.95</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>21.40599792764294</v>
+        <v>21.40599791954565</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>44.26588943665861</v>
+        <v>44.26588948936259</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.7874626120692589</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.5309074311090769</v>
+        <v>-0.5309074312388617</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>39.73776973152281</v>
+        <v>39.73776979145151</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.40623331286562</v>
+        <v>19.40623334405278</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3077231608524913</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.429248590160621</v>
+        <v>-1.429248591017228</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>216.5822191338144</v>
+        <v>216.582219133814</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>926</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>37.54317172077666</v>
+        <v>37.54317166423133</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.0232836516637</v>
+        <v>16.02328364535037</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.5343834419098776</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-18.76718774738901</v>
+        <v>-18.7671877414189</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>215.757693736051</v>
+        <v>215.7576937360512</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>40.1</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>38.56828214230803</v>
+        <v>38.56828228591925</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>17.10038958283439</v>
+        <v>17.10038947967988</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8576656281890479</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.1217869542394101</v>
+        <v>-0.1217869545119623</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>214.080037949927</v>
+        <v>214.0800379499272</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>40.5</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>26.28913536482523</v>
+        <v>26.28913556583321</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>26.54801594809214</v>
+        <v>26.54801599183065</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>2.949319726682562</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.3661010551668421</v>
+        <v>-0.3661010557898211</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>43.34250961382213</v>
+        <v>43.34250966330838</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.68292009356607</v>
+        <v>15.68292024058454</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.8438653737703994</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.2705272734237828</v>
+        <v>-0.2705272740727045</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>200.9505152553307</v>
+        <v>200.9505152553305</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>265.5</v>
@@ -5484,7 +5484,7 @@
         <v>43.41569628885242</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.67901079375986</v>
+        <v>14.67901080419101</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.6326269508565294</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.9047023276277858</v>
+        <v>-0.9047023278873767</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>199.4382712759071</v>
+        <v>199.4382712759072</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>82</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>40.09180236856827</v>
+        <v>40.09180249583243</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>24.41660655924312</v>
+        <v>24.41660680609541</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.5064801776707681</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-1.048188103617851</v>
+        <v>-1.048188104656152</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>197.1715355105348</v>
+        <v>197.1715355105349</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>4795</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.2762972986605</v>
+        <v>33.27629725311847</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.97865290202665</v>
+        <v>14.97865287448744</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.6564747559939048</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-72.64529324250736</v>
+        <v>-72.64529320746504</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>36.56913230109119</v>
+        <v>36.56913232718083</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>13.95121355982481</v>
+        <v>13.95121362415139</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2295559865264877</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.3092166365498175</v>
+        <v>-0.3092166364979061</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>33.71677436391838</v>
+        <v>33.71677435045174</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>17.41840566827861</v>
+        <v>17.41840568889002</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.9639672741997238</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.7233282320283039</v>
+        <v>-0.7233282320542629</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.23265772565979</v>
+        <v>38.23265781965636</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.10840643560025</v>
+        <v>14.10840660540173</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.6871211123918444</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.6547386059153331</v>
+        <v>-0.6547386077323591</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>175.4387437829409</v>
+        <v>175.438743782941</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>859</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>30.84331241236315</v>
+        <v>30.84331244071844</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>17.51079320512153</v>
+        <v>17.51079325931505</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.9455860644478375</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-23.3572199312885</v>
+        <v>-23.35721993622049</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.66054429092895</v>
+        <v>41.66054431127788</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>11.63473792414037</v>
+        <v>11.63473806286067</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.426879794646962</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.975618231375056</v>
+        <v>-0.9756182318422915</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>173.2149216876153</v>
+        <v>173.2149216876154</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>14.9</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>34.52698748010312</v>
+        <v>34.52698758375153</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.85300313781395</v>
+        <v>12.85300329214043</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5863412207844794</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.06683297948937778</v>
+        <v>-0.06683297958023071</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>173.127452659446</v>
+        <v>173.1274526594421</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>42.9</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>47.97269727529312</v>
+        <v>47.97269723269763</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>22.52746597995064</v>
+        <v>22.52746607353626</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6526611454951174</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1675612827556942</v>
+        <v>-0.1675612828595288</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>171.9884022078905</v>
+        <v>171.9884022078907</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>62.8</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.97715400040907</v>
+        <v>42.97715411530697</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.97409217320356</v>
+        <v>18.97409229374122</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.7867980004608999</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.01147898376756806</v>
+        <v>-0.01147898441650158</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.71532878835846</v>
+        <v>39.71532844214489</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>24.30403332458481</v>
+        <v>24.30403280657199</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.9455693773517216</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.008969119555023941</v>
+        <v>-0.008969119373324452</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>167.5560185719689</v>
+        <v>167.5560185719671</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>183.5</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>27.89453628424448</v>
+        <v>27.89453630995776</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>22.01073616536327</v>
+        <v>22.01073610534473</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.8252017209539247</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-2.232520024227547</v>
+        <v>-2.232520028640305</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>154.785698155389</v>
+        <v>154.7856981554012</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>41</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>37.31586480749338</v>
+        <v>37.31586533971147</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>26.36153818669313</v>
+        <v>26.36153766379905</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.318412413675747</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.141117210436248</v>
+        <v>-0.141117213525174</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>152.3622198772974</v>
+        <v>152.3622198772971</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>34.75</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>36.62982868931608</v>
+        <v>36.62982858532308</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>17.49897958363209</v>
+        <v>17.49897958078801</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.363175764211213</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.03247424250219594</v>
+        <v>-0.03247424245027758</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>151.7255347205413</v>
+        <v>151.7255347205412</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>32</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>38.35913983955815</v>
+        <v>38.3591398493494</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>13.93194917199847</v>
+        <v>13.93194927861356</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.7759780660098581</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1125227123663517</v>
+        <v>-0.1125227124961461</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>148.5276620730933</v>
+        <v>148.5276620730914</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>344.5</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>45.18383023507294</v>
+        <v>45.18383036083535</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>15.66093060959008</v>
+        <v>15.66093050789494</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.9699175223982399</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-1.660841262628599</v>
+        <v>-1.660841267300894</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>145.7432013221261</v>
+        <v>145.7432013221235</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>58</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>36.31898698664166</v>
+        <v>36.31898703426123</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.16895049079034</v>
+        <v>14.16895044921982</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>1.450468926701203</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.5018539236248256</v>
+        <v>-0.5018539221452558</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>44.53992713661643</v>
+        <v>44.53992733313947</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>10.7207042710617</v>
+        <v>10.7207044319531</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.220558012629307</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.3022272982951256</v>
+        <v>-0.3022272994632306</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>36.96824743716958</v>
+        <v>36.96824750946424</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.99138118783948</v>
+        <v>17.99138129048388</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6584490444323197</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.111386877686469</v>
+        <v>-0.1113868779330675</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>133.6386667029438</v>
+        <v>133.6386667029439</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>0</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>43.86676874263865</v>
+        <v>43.86676874555715</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>7.916759231856679</v>
+        <v>7.91675924262438</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.03182800231859619</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-3.604103287005568</v>
+        <v>-3.604103287862157</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>128.5920057126307</v>
+        <v>128.5920057126382</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>22.8</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>34.77941121713503</v>
+        <v>34.77941199701893</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>20.72033330455541</v>
+        <v>20.72033330012372</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.924548321422329</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1755610842121617</v>
+        <v>-0.1755610848870561</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>36.79184445666461</v>
+        <v>36.79184456781395</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.09987930055115</v>
+        <v>12.09987951456267</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.265351474409393</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.3918666922667249</v>
+        <v>-0.3918666935645807</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>118.2576117047335</v>
+        <v>118.2576117047331</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>21.8</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>47.26288422599929</v>
+        <v>47.26288429019858</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>5.795790550401364</v>
+        <v>5.795790529757819</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>1.122671959263046</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.06240903961362998</v>
+        <v>-0.06240903966554397</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>112.1983040126149</v>
+        <v>112.198304012618</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>46.4</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>30.00378459078681</v>
+        <v>30.00378456922876</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.7706306745425</v>
+        <v>17.77063087317586</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.7359613321447603</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.3541510675606661</v>
+        <v>-0.3541510675347144</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>102.3778883402266</v>
+        <v>102.3778883402265</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>51</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>35.23191218394592</v>
+        <v>35.23191201543608</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>16.99568485809011</v>
+        <v>16.9956848580901</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.7207567279509726</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.2627715875734209</v>
+        <v>-0.2627715872100173</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>33.88921851522797</v>
+        <v>33.88921839162201</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>18.30733162818931</v>
+        <v>18.30733187662078</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.9540766572628137</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.2731121999218314</v>
+        <v>-0.2731121999737434</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>35.39904265510241</v>
+        <v>35.39904266783469</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>19.17178749502515</v>
+        <v>19.17178754028631</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.2556153940612024</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.2689371536185194</v>
+        <v>-0.2689371536963937</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>52.14023492167311</v>
+        <v>52.1402346940598</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>9.353446190962234</v>
+        <v>9.353446199014604</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.3514335018088489</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-2.122319380446635</v>
+        <v>-2.122319380213018</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>32.211578936419</v>
+        <v>32.21157909710476</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>14.55094407722806</v>
+        <v>14.55094398558052</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>1.394987601904179</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.1025562344087536</v>
+        <v>-0.1025562348759875</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>50.41842289188457</v>
+        <v>50.41842289188414</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>185</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>33.93692737920014</v>
+        <v>33.93692755281964</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18.13702678523131</v>
+        <v>18.13702697844792</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.4194506896377507</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.048898902873951</v>
+        <v>-1.048898904820752</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg6 2026-10-27 00:08 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq7_2026-10-22.xlsx
@@ -552,7 +552,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>66.1392107296813</v>
+        <v>66.13921086902906</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>38.17180869844601</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.3898117225347661</v>
+        <v>0.3898117216937216</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>67.99301297688395</v>
+        <v>67.99301300452638</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>33.76309485096934</v>
+        <v>33.76309483082886</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.16131508790875</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.909568498481043</v>
+        <v>2.909568499322045</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>59.43460131000813</v>
+        <v>59.4346013253661</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>32.95138991962353</v>
+        <v>32.95138993494632</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.8531135934803761</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.3295393344551192</v>
+        <v>0.3295393359969534</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.45357812491665</v>
+        <v>65.45357822397415</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>42.47737231439886</v>
+        <v>42.47737234107753</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0.9817295434887761</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.9360722867009024</v>
+        <v>0.9360722851590673</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>59.26265219171178</v>
+        <v>59.26265229279267</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23.43592318906657</v>
+        <v>23.43592322032801</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.590262182470743</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.4499754969948003</v>
+        <v>0.4499754967424964</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>78.84064557796489</v>
+        <v>78.84064559801708</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>28.03469086900749</v>
+        <v>28.03469088502624</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.805710472882409</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3.452091477314043</v>
+        <v>3.452091477398128</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>53.54270783774406</v>
+        <v>53.5427078944462</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>33.66656639386537</v>
+        <v>33.66656644912623</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.6014135830005847</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-8.764929627189638</v>
+        <v>-8.764929629712732</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65.62661536859808</v>
+        <v>65.62661538343271</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>62.72758505166355</v>
+        <v>62.72758511805647</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.016111572061801</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>4.675131238420221</v>
+        <v>4.675131238139826</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>707.6393411866211</v>
+        <v>707.6393411866203</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>30.3</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>66.18319005050003</v>
+        <v>66.18319010800732</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>18.52913199507876</v>
+        <v>18.52913194966825</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.639202115466247</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2807110429230415</v>
+        <v>0.2807110430211575</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>52.83820016037561</v>
+        <v>52.83820013835843</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>27.7481548157389</v>
+        <v>27.74815497667672</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.7489979191491927</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-14.9542763334002</v>
+        <v>-14.95427633760524</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>54.83324439600781</v>
+        <v>54.83324440047032</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>57.22228095341231</v>
+        <v>57.22228089967729</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.8508086301746604</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.870886421714447</v>
+        <v>-0.8708864218265724</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>58.46748228248495</v>
+        <v>58.46748230062387</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>29.42322241829411</v>
+        <v>29.42322235124522</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.4228143041877703</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.2813739006544933</v>
+        <v>-0.2813739005283402</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>54.44818794517776</v>
+        <v>54.44818796187293</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>30.82920264781097</v>
+        <v>30.82920265758897</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.9635624771200302</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-5.137034638345732</v>
+        <v>-5.137034639326931</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>43.35024341425321</v>
+        <v>43.3502434232258</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>27.30615659592426</v>
+        <v>27.30615662781592</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.5381821608099771</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-9.710584682508859</v>
+        <v>-9.710584682957355</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.8626354899997</v>
+        <v>51.86263549805991</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>48.28267928124164</v>
+        <v>48.28267964092949</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.569845152521627</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-1.284393853309933</v>
+        <v>-1.284393853478118</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>50.18528360302879</v>
+        <v>50.18528362518579</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>39.06509014432356</v>
+        <v>39.06509015990518</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4366239614420854</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-1.414578922880661</v>
+        <v>-1.41457892318904</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46.79904153805073</v>
+        <v>46.79904147356019</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15.97781209733668</v>
+        <v>15.97781214399657</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.7493361150785418</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-15.217724242888</v>
+        <v>-15.2177242316742</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>43.07886121885245</v>
+        <v>43.07886110743026</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.76290932082123</v>
+        <v>23.76290945321622</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.4024984031592331</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-11.26967931414019</v>
+        <v>-11.26967931007528</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>68.41252470798648</v>
+        <v>68.41252472060631</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>36.2393281840283</v>
+        <v>36.23932822668347</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.71445693349921</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>1.09213665188584</v>
+        <v>1.092136651857801</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>53.34021960790697</v>
+        <v>53.34021962875246</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>46.52032367085199</v>
+        <v>46.5203236614463</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.6871215099514526</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.437477560446089</v>
+        <v>-0.437477560418051</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.48352346686449</v>
+        <v>51.48352350424349</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>50.23478175815763</v>
+        <v>50.23478191509314</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.6979013411604504</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.2186659814809033</v>
+        <v>-0.2186659813547429</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>31.69503670044691</v>
+        <v>31.69497250770478</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>32.59384563926454</v>
+        <v>32.59385527628714</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>2.013053626871307</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.4112800741141505</v>
+        <v>0.4112802541172318</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>44.81020338410932</v>
+        <v>44.81020339441604</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>40.69951900598078</v>
+        <v>40.69951901745065</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.4716996868395078</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-2.284573293188202</v>
+        <v>-2.284573293328349</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>502.5889994943347</v>
+        <v>502.5889994943348</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>311.5</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>47.37589240126501</v>
+        <v>47.37589244330629</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>14.92085526119895</v>
+        <v>14.92085530658707</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.106793234680007</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.7874918208919892</v>
+        <v>0.787491821032134</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.38347057721097</v>
+        <v>51.3834706934419</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>27.49474112937997</v>
+        <v>27.49474123505709</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7258430839794561</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.4625791000991539</v>
+        <v>0.4625790998748784</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>54.78509626425939</v>
+        <v>54.78509628062488</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>27.82618267411424</v>
+        <v>27.82618274896065</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.132039438032072</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.9246587924377483</v>
+        <v>-0.9246587927180876</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>53.56737410844026</v>
+        <v>53.56737411351146</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>9.652436801055186</v>
+        <v>9.652436801055183</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.2573020601650947</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2.051568861311428</v>
+        <v>2.051568861031096</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.34519241469733</v>
+        <v>56.34519243255516</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.056540362229</v>
+        <v>28.05654046689048</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.025511535086557</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.1872518385968903</v>
+        <v>0.1872518385688512</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>476.4333302809613</v>
+        <v>476.4333302809612</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>54.6</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>52.88280168553795</v>
+        <v>52.88280199326524</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>5.805252003337797</v>
+        <v>5.805252004910519</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>7.041140377347645</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>52.0556434529181</v>
+        <v>52.05564341145131</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.2986858100039</v>
+        <v>26.29868579549269</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.8608248155283107</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.01786095505396873</v>
+        <v>-0.01786095496986972</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>472.113715946996</v>
+        <v>472.1137159469962</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>252</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.82436370508728</v>
+        <v>44.82436400897409</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.81613439668219</v>
+        <v>31.81613426493104</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.3268196648928203</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-3.159187638148364</v>
+        <v>-3.159187641932927</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>43.73114175639572</v>
+        <v>43.73114175999579</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.34487843277425</v>
+        <v>26.34487846868186</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.6504221412525585</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.5703199971067308</v>
+        <v>-0.5703199970786987</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>56.3009077493245</v>
+        <v>56.30090773721639</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>51.76728172823847</v>
+        <v>51.76728185570251</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.7293381745137858</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.5204985936455411</v>
+        <v>-0.5204985932250343</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>43.03381971953389</v>
+        <v>43.03381972959243</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>12.36682424409357</v>
+        <v>12.36682429327928</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.083874176340649</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.8400575301784277</v>
+        <v>-0.8400575302765469</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>43.1835045825207</v>
+        <v>43.18350464483397</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>12.40643357572483</v>
+        <v>12.40643355901833</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6707571425321006</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.2985029117954729</v>
+        <v>-0.2985029113749809</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>430.2730399096475</v>
+        <v>430.2730399096472</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>33.35</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>51.72229192552977</v>
+        <v>51.72229193474445</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>9.070079142315496</v>
+        <v>9.070079207256374</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.3094123228614452</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.6731305966550249</v>
+        <v>0.6731305964868235</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>426.6714799216026</v>
+        <v>426.6714799216048</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>438</v>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>43.4631689606963</v>
+        <v>43.46316894079558</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>16.89368721941255</v>
+        <v>16.89368720997794</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.345272722820805</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-3.835548446912627</v>
+        <v>-3.835548446071636</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>408.0379727000433</v>
+        <v>408.0379727000432</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>200</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46.49124106814377</v>
+        <v>46.49124107787478</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>24.1584157632592</v>
+        <v>24.15841581507631</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3055407865693525</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-2.150556973750456</v>
+        <v>-2.150556974311132</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>405.7485851320556</v>
+        <v>405.7485851320558</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>20.25</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>51.94049266350598</v>
+        <v>51.94049266836732</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>7.008649904222151</v>
+        <v>7.008649904222149</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.2940991325586373</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.4766114651531362</v>
+        <v>0.4766114650970712</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.95463226293367</v>
+        <v>66.95463310228067</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>45.75795694778152</v>
+        <v>45.75795718842983</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.02373845207331912</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.08210771244663961</v>
+        <v>-0.08210771272697814</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>35.84716741032861</v>
+        <v>35.84716736347902</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>17.17900475190858</v>
+        <v>17.17900478612803</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.089224249952527</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-4.485548443541893</v>
+        <v>-4.48554844129916</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
         <v>46.20316293156278</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>24.30802590981961</v>
+        <v>24.30802597102479</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.8379661521848411</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>48.30030412799786</v>
+        <v>48.30030421339518</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>18.16462395776582</v>
+        <v>18.16462392961186</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.5443416099734087</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.2480839149300026</v>
+        <v>-0.2480839149019693</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>375.2572561347595</v>
+        <v>375.2572561347596</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>101</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>40.09459933619632</v>
+        <v>40.09459930206293</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>18.99730027605282</v>
+        <v>18.9973003499917</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.1878142965022349</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-1.404968961968843</v>
+        <v>-1.404968960847497</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>57.95102201636346</v>
+        <v>57.95102199505163</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>31.95665076381545</v>
+        <v>31.95665095813985</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.3298076254041656</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.1895555951710248</v>
+        <v>-0.1895555950375651</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>46.72811523788231</v>
+        <v>46.72811538826433</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>11.26984672375984</v>
+        <v>11.26984670537118</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6769276009064168</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.01091292296101987</v>
+        <v>-0.01091292307315744</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>48.32045144933695</v>
+        <v>48.32045146900536</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>31.32192080889711</v>
+        <v>31.32192082065117</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.2662409917239372</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.10941825648063</v>
+        <v>-1.109418256592772</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>360.4100534133018</v>
+        <v>360.4100534133017</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>78.90000000000001</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>43.56709064958579</v>
+        <v>43.56709061264517</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>10.08296175367835</v>
+        <v>10.08296169768746</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>2.549799792792541</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.1478458583582646</v>
+        <v>-0.1478458583862963</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>356.9683100161362</v>
+        <v>356.9683100161369</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>31.5</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.92650940199975</v>
+        <v>48.92650955845977</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.99380493462421</v>
+        <v>19.99380504451578</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5109288470936049</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.02340443989559124</v>
+        <v>0.02340443976944023</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.99051756841304</v>
+        <v>42.9905176116556</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>20.66308834710163</v>
+        <v>20.66308839321755</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.3495772391539256</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-8.014021952917089</v>
+        <v>-8.01402195235644</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>38.18810824051624</v>
+        <v>38.188108279048</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>17.91025758856495</v>
+        <v>17.9102577063196</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.7056395626210019</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-20.78787311305849</v>
+        <v>-20.78787311586193</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>33.17659636557011</v>
+        <v>33.1765967386052</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>20.26534206916199</v>
+        <v>20.26534232195076</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5502769291013172</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.089700698283113</v>
+        <v>0.08970069772243372</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>35.37096399870065</v>
+        <v>35.3709640165477</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.63443392768182</v>
+        <v>19.6344339160425</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4854669172735663</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-4.725979832839229</v>
+        <v>-4.725979832699077</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>342.510162472793</v>
+        <v>342.5101624727927</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>13.65</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.50275291412495</v>
+        <v>52.50275305108977</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>32.03331397758119</v>
+        <v>32.03331399513685</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.2502473810573438</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.04269046727003761</v>
+        <v>0.04269046717191888</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>341.6518351144287</v>
+        <v>341.6518351144687</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>32.45</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.58701152949315</v>
+        <v>44.58701224867362</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>34.91832383570953</v>
+        <v>34.91832393002793</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6421649717445593</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.06698707021551151</v>
+        <v>-0.0669870704678196</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>49.07558613941439</v>
+        <v>49.07558608658073</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.76965326559563</v>
+        <v>29.76965336574128</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.2095738242586338</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0147037856488178</v>
+        <v>0.01470378573291775</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>337.2072573496719</v>
+        <v>337.2072573496715</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>91.2</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>45.57284605879392</v>
+        <v>45.5728460944547</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22.30864813798438</v>
+        <v>22.30864830335075</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.3985145381141949</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.2983714169664006</v>
+        <v>-0.2983714171065608</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>34.22897735258211</v>
+        <v>34.22897740857138</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.73589107735793</v>
+        <v>20.73589106703014</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.9734623319790414</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-8.648725455973132</v>
+        <v>-8.648725456814125</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>41.14913936781046</v>
+        <v>41.14913964405964</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>25.72357658324564</v>
+        <v>25.7235765978812</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.402942734216557</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.1216434035570048</v>
+        <v>0.1216434034728995</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>53.44229464300494</v>
+        <v>53.44229490888937</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.6320224634039</v>
+        <v>11.63202241564493</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.8362066563706447</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.08618012212925803</v>
+        <v>0.08618012198908881</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>32.50477980118534</v>
+        <v>32.50477979485358</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>23.76985613690461</v>
+        <v>23.76985618398827</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4050616365577276</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-2.111207928976355</v>
+        <v>-2.111207928934308</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.95815849138076</v>
+        <v>45.9581585663008</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.62736460384406</v>
+        <v>23.62736462748841</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.2951796718019397</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-8.083918670691094</v>
+        <v>-8.083918669990254</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>316.1874022349516</v>
+        <v>316.1874022349515</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>30.25</v>
@@ -3841,7 +3841,7 @@
         <v>43.44051007368235</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.19302544013198</v>
+        <v>15.19302546784974</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.5672759078947981</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.02873342428836156</v>
+        <v>0.02873342423229253</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>32.35210813950101</v>
+        <v>32.35210815829876</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>16.34739219273574</v>
+        <v>16.34739210388565</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8197253114347555</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.805532682131642</v>
+        <v>-1.805532681739159</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>27.72976066393656</v>
+        <v>27.72976065372578</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>42.34235323582792</v>
+        <v>42.34235323300104</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.004128314746851</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>75.32137559096594</v>
+        <v>75.3213756049829</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>297.7362003466068</v>
+        <v>297.7362003466066</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>260</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>34.33551212391791</v>
+        <v>34.33551219180684</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>27.29241267166761</v>
+        <v>27.29241261708051</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.836939751452674</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.2469649439947585</v>
+        <v>-0.2469649441349024</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>29.52310241874801</v>
+        <v>29.52310234376185</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>25.68840367579241</v>
+        <v>25.68840366218092</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.200584827670398</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-9.807987038093273</v>
+        <v>-9.807987036691539</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>279.0374276364245</v>
+        <v>279.0374276364252</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>72.5</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>38.43366142992564</v>
+        <v>38.43366171091558</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>13.86832634216873</v>
+        <v>13.86832628411494</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.7472854498730647</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.03638324395258907</v>
+        <v>-0.03638324431701956</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>277.7385177368528</v>
+        <v>277.7385177368533</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>395.5</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>28.43930784168762</v>
+        <v>28.43930790118735</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>35.7744994488714</v>
+        <v>35.77449953462034</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7541966637473086</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-4.238642015778581</v>
+        <v>-4.23864201605894</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>277.3596224343956</v>
+        <v>277.3596224343964</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>58.3</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>43.39129164622928</v>
+        <v>43.39129141881397</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>35.56974151595632</v>
+        <v>35.56974182774109</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6387248817360134</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1680993623833887</v>
+        <v>-0.1680993613181026</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>276.9361253032197</v>
+        <v>276.9361253032192</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>31.7</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>47.67833461021966</v>
+        <v>47.67833490598038</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>9.78895211616444</v>
+        <v>9.788952076536136</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.5970128778915239</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.1662612070594894</v>
+        <v>-0.1662612066389842</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>276.9119108428752</v>
+        <v>276.911910842875</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>149.5</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>46.02335630685144</v>
+        <v>46.02335722870358</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.4462165566942</v>
+        <v>14.44621653929905</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7434437233323928</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.05975606739983655</v>
+        <v>-0.0597560678203484</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>29.22695765456382</v>
+        <v>29.22695770150469</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>27.55583681127679</v>
+        <v>27.55583686584252</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.7308142214645494</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.458553579185219</v>
+        <v>-1.458553580306575</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>275.0239908494917</v>
+        <v>275.0239908494918</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>441</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>26.46661251627982</v>
+        <v>26.4666126343879</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>29.81781723267084</v>
+        <v>29.81781727896692</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.8925733520485345</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-6.633611730725779</v>
+        <v>-6.63361173493087</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>268.1452942390133</v>
+        <v>268.1452942390119</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>45.8</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>40.84354946040339</v>
+        <v>40.84355003935577</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>18.4414987393686</v>
+        <v>18.44149884932769</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.5938828997542779</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.3072017301711005</v>
+        <v>-0.3072017307598105</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>263.0778103664687</v>
+        <v>263.0778103664711</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>30.7</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>44.23307551790457</v>
+        <v>44.23307550303868</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>10.22886681524779</v>
+        <v>10.22886682112144</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4323671099305398</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.0182686383042428</v>
+        <v>-0.01826863806595541</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>259.9620847677766</v>
+        <v>259.9620847677765</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>120</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>24.94382259600208</v>
+        <v>24.94382378046984</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>25.98054366655018</v>
+        <v>25.98054392934254</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.8455976587157367</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.6673542159617645</v>
+        <v>-0.6673542173634717</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>48.58712143966925</v>
+        <v>48.58712142593199</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>8.315858922171255</v>
+        <v>8.315858962698215</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.500846362264681</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.02764861326743581</v>
+        <v>-0.02764861329547069</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4689,7 +4689,7 @@
         <v>44.84000589582177</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>11.71674973081112</v>
+        <v>11.71674977110114</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.334053863089634</v>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>244.4507352996496</v>
+        <v>244.450735299649</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>22.7</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>43.29872271509428</v>
+        <v>43.29872296846128</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13.85678704041722</v>
+        <v>13.85678703855465</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1.862922723609504</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.002855709708819942</v>
+        <v>0.002855709596684013</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>47.19009974328522</v>
+        <v>47.19009969851058</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>46.63856802785586</v>
+        <v>46.63856822558206</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4126321019762629</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.11169780820985</v>
+        <v>-0.1116978080836957</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>228.3106571009501</v>
+        <v>228.31065710095</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>1185</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>36.06335611145087</v>
+        <v>36.06335610028396</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.79376418230428</v>
+        <v>15.79376415287457</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.3608053483989695</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-35.14971342308185</v>
+        <v>-35.14971342322215</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>46.68799822251765</v>
+        <v>46.68799830454859</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>14.64900051592594</v>
+        <v>14.64900059175885</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3262171362946557</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.03055587933814333</v>
+        <v>0.03055587929609183</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>221.8527820116686</v>
+        <v>221.8527820116681</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>144.5</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>27.60894648873207</v>
+        <v>27.60894699229392</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>25.30617069015616</v>
+        <v>25.30617073126552</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.9479146470974632</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-1.598952410509593</v>
+        <v>-1.598952410089106</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>221.1790849490206</v>
+        <v>221.1790849490193</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>52.6</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>41.77962525496796</v>
+        <v>41.77962540882611</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.08018110625801</v>
+        <v>12.08018113045676</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.8521506427035332</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.01195447589739312</v>
+        <v>-0.01195447570115132</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>35.2925568095651</v>
+        <v>35.29255685708418</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>20.52550766544719</v>
+        <v>20.5255077835756</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.6771364144255658</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-31.71910485106393</v>
+        <v>-31.71910485344681</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>29.57274247949711</v>
+        <v>29.57274270797694</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>38.79309213470124</v>
+        <v>38.79309203501879</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.726196054107507</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.4162327281921847</v>
+        <v>-0.4162327286127092</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>21.40599791954565</v>
+        <v>21.40599799809155</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>44.26588948936259</v>
+        <v>44.26588953336294</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.7874626120692589</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.5309074312388617</v>
+        <v>-0.5309074314350966</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>216.6774747195185</v>
+        <v>216.6774747195184</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>87</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>39.73776979145151</v>
+        <v>39.73776981771555</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.40623334405278</v>
+        <v>19.40623334707202</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3077231608524913</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.429248591017228</v>
+        <v>-1.429248591073291</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>216.582219133814</v>
+        <v>216.5822191338143</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>926</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>37.54317166423133</v>
+        <v>37.54317165735252</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.02328364535037</v>
+        <v>16.02328364322718</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.5343834419098776</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-18.7671877414189</v>
+        <v>-18.76718774310074</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>215.7576937360512</v>
+        <v>215.7576937360513</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>40.1</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>38.56828228591925</v>
+        <v>38.5682822049078</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>17.10038947967988</v>
+        <v>17.10038945604524</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8576656281890479</v>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>214.0800379499272</v>
+        <v>214.0800379499271</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>40.5</v>
@@ -5375,7 +5375,7 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>26.28913556583321</v>
+        <v>26.28913581491881</v>
       </c>
       <c r="I93" s="2" t="n">
         <v>26.54801599183065</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.3661010557898211</v>
+        <v>-0.3661010557617848</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>43.34250966330838</v>
+        <v>43.34250983050352</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.68292024058454</v>
+        <v>15.68292030705092</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.8438653737703994</v>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>200.9505152553305</v>
+        <v>200.9505152553301</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>265.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>43.41569628885242</v>
+        <v>43.41569638667294</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.67901080419101</v>
+        <v>14.67901089273067</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.6326269508565294</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.9047023278873767</v>
+        <v>-0.9047023281677411</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>199.4382712759072</v>
+        <v>199.4382712759071</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>82</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>40.09180249583243</v>
+        <v>40.09180256849511</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>24.41660680609541</v>
+        <v>24.41660683787188</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.5064801776707681</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-1.048188104656152</v>
+        <v>-1.048188104880418</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>197.1715355105349</v>
+        <v>197.1715355105348</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>4795</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.27629725311847</v>
+        <v>33.2762972553478</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.97865287448744</v>
+        <v>14.97865286691651</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.6564747559939048</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-72.64529320746504</v>
+        <v>-72.64529320045665</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>190.4094290413522</v>
+        <v>190.409429041352</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>68.59999999999999</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>36.56913232718083</v>
+        <v>36.56913229908429</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>13.95121362415139</v>
+        <v>13.95121374805123</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2295559865264877</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.3092166364979061</v>
+        <v>-0.3092166363577347</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>33.71677435045174</v>
+        <v>33.71677439709018</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>17.41840568889002</v>
+        <v>17.41840578596958</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.9639672741997238</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.7233282320542629</v>
+        <v>-0.7233282321944221</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.23265781965636</v>
+        <v>38.2326580273229</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>14.10840660540173</v>
+        <v>14.10840663123291</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.6871211123918444</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.6547386077323591</v>
+        <v>-0.654738608012698</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>30.84331244071844</v>
+        <v>30.84331243228687</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>17.51079325931505</v>
+        <v>17.51079329445206</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.9455860644478375</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-23.35721993622049</v>
+        <v>-23.35721993565985</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>175.0969944387909</v>
+        <v>175.0969944387908</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>137</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.66054431127788</v>
+        <v>41.66054437593844</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>11.63473806286067</v>
+        <v>11.63473815996391</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.426879794646962</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.9756182318422915</v>
+        <v>-0.9756182320104847</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>34.52698758375153</v>
+        <v>34.52698753418471</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.85300329214043</v>
+        <v>12.8530033683571</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5863412207844794</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.06683297958023071</v>
+        <v>-0.06683297955219725</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>47.97269723269763</v>
+        <v>47.97269733288427</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>22.52746607353626</v>
+        <v>22.52746597826046</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6526611454951174</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1675612828595288</v>
+        <v>-0.1675612831819193</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>171.9884022078907</v>
+        <v>171.9884022078905</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>62.8</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.97715411530697</v>
+        <v>42.97715423904318</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.97409229374122</v>
+        <v>18.97409233677135</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.7867980004608999</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.01147898441650158</v>
+        <v>-0.01147898483701068</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.71532844214489</v>
+        <v>39.71532864325808</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>24.30403280657199</v>
+        <v>24.30403328499385</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.9455693773517216</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.008969119373324452</v>
+        <v>-0.008969119583579488</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>27.89453630995776</v>
+        <v>27.89453646304345</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>22.01073610534473</v>
+        <v>22.01073604144524</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.8252017209539247</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-2.232520028640305</v>
+        <v>-2.232520032565056</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>154.7856981554012</v>
+        <v>154.7856981553956</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>41</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>37.31586533971147</v>
+        <v>37.31586667069898</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>26.36153766379905</v>
+        <v>26.36153708458932</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.318412413675747</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.141117213525174</v>
+        <v>-0.1411172154034539</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>36.62982858532308</v>
+        <v>36.62982829401579</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>17.49897958078801</v>
+        <v>17.49897962427012</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.363175764211213</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>38.3591398493494</v>
+        <v>38.35914017110695</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>13.93194927861356</v>
+        <v>13.93194944378122</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.7759780660098581</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1125227124961461</v>
+        <v>-0.1125227126082735</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>148.5276620730914</v>
+        <v>148.5276620730938</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>344.5</v>
@@ -6332,7 +6332,7 @@
         <v>45.18383036083535</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>15.66093050789494</v>
+        <v>15.66093048955033</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.9699175223982399</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-1.660841267300894</v>
+        <v>-1.660841267020589</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>145.7432013221235</v>
+        <v>145.7432013221246</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>58</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>36.31898703426123</v>
+        <v>36.31898663254755</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.16895044921982</v>
+        <v>14.16895059412443</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>1.450468926701203</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.5018539221452558</v>
+        <v>-0.5018539203791148</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
         <v>44.53992733313947</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>10.7207044319531</v>
+        <v>10.7207044470847</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.220558012629307</v>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>139.9667786670803</v>
+        <v>139.9667786670809</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>23.1</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>36.96824750946424</v>
+        <v>36.96824771607542</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.99138129048388</v>
+        <v>17.99138144463401</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6584490444323197</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1113868779330675</v>
+        <v>-0.1113868780872527</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>43.86676874555715</v>
+        <v>43.86676874914795</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>7.91675924262438</v>
+        <v>7.916759228392235</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.03182800231859619</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-3.604103287862157</v>
+        <v>-3.604103288338736</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>128.5920057126382</v>
+        <v>128.5920057126358</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>22.8</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>34.77941199701893</v>
+        <v>34.7794114241959</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>20.72033330012372</v>
+        <v>20.72033331917374</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.924548321422329</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1755610848870561</v>
+        <v>-0.1755610843824418</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>36.79184456781395</v>
+        <v>36.79184482475628</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.09987951456267</v>
+        <v>12.09987961944049</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.265351474409393</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.3918666935645807</v>
+        <v>-0.3918666939850907</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>118.2576117047331</v>
+        <v>118.2576117047334</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>21.8</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>47.26288429019858</v>
+        <v>47.26288423515511</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>5.795790529757819</v>
+        <v>5.79579051840313</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>1.122671959263046</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.06240903966554397</v>
+        <v>-0.06240903946930922</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>30.00378456922876</v>
+        <v>30.00378457831442</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.77063087317586</v>
+        <v>17.77063088087114</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.7359613321447603</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.3541510675347144</v>
+        <v>-0.3541510675767627</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>102.3778883402265</v>
+        <v>102.3778883402266</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>51</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>35.23191201543608</v>
+        <v>35.2319120449565</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>16.9956848580901</v>
+        <v>16.99568481957185</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.7207567279509726</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.2627715872100173</v>
+        <v>-0.2627715873501861</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>99.31000499851136</v>
+        <v>99.31000499851125</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>56.8</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>33.88921839162201</v>
+        <v>33.88921848670353</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>18.30733187662078</v>
+        <v>18.30733185540374</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.9540766572628137</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.2731121999737434</v>
+        <v>-0.2731122006185274</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6915,7 +6915,7 @@
         <v>35.39904266783469</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>19.17178754028631</v>
+        <v>19.17178760395885</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.2556153940612024</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.2689371536963937</v>
+        <v>-0.2689371537524581</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>52.1402346940598</v>
+        <v>52.14023514444288</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>9.353446199014604</v>
+        <v>9.353447453733999</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.3514335018088489</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-2.122319380213018</v>
+        <v>-2.122319390291233</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>32.21157909710476</v>
+        <v>32.21157935107789</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>14.55094398558052</v>
+        <v>14.55094390011431</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>1.394987601904179</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.1025562348759875</v>
+        <v>-0.1025562351282898</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>50.41842289188414</v>
+        <v>50.41842289188371</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>185</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>33.93692755281964</v>
+        <v>33.93692758775001</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18.13702697844792</v>
+        <v>18.13702703594532</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.4194506896377507</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.048898904820752</v>
+        <v>-1.048898904400262</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>

</xml_diff>